<commit_message>
updated flexible dimensions, contract type for ValueVariable
</commit_message>
<xml_diff>
--- a/data/dimensions/dimensions.xlsx
+++ b/data/dimensions/dimensions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GIT\cross_back\initial_data\classifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9437E5C-718D-41CA-B2A9-2CCBCB9F117F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303C2C7F-FCCE-457C-8507-2B20BC5AA717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="1080" windowWidth="30900" windowHeight="14460" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="21" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2218" uniqueCount="1339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2218" uniqueCount="1338">
   <si>
     <t>id</t>
   </si>
@@ -3368,9 +3368,6 @@
   </si>
   <si>
     <t>variant</t>
-  </si>
-  <si>
-    <t>explanation</t>
   </si>
   <si>
     <t>abroad-together</t>
@@ -4478,176 +4475,176 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>1272</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>1273</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>1274</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>1275</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>1276</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
+        <v>1276</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>1277</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1278</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>1279</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>1280</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1281</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
+        <v>1282</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>1283</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1284</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
+        <v>1284</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>1285</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1286</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>1288</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1289</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>1291</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>1292</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
+        <v>1293</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>1294</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>1295</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
+        <v>1296</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>1297</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>1298</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
+        <v>1299</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>1300</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>1301</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>1303</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>1304</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>1305</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>1306</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
   </sheetData>
@@ -8292,148 +8289,148 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
+        <v>1306</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>1307</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>1308</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>1309</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>1106</v>
       </c>
       <c r="F1" s="7" t="s">
+        <v>1309</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>1310</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>1311</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>1312</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>1313</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>1314</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>1315</v>
       </c>
       <c r="D2" s="7">
         <v>2020</v>
       </c>
       <c r="F2" s="7" t="s">
+        <v>1315</v>
+      </c>
+      <c r="G2" s="7" t="s">
         <v>1316</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="5" t="s">
         <v>1317</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>1318</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>1319</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>1320</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>1321</v>
       </c>
       <c r="D3" s="7">
         <v>2017</v>
       </c>
       <c r="E3" s="7" t="s">
+        <v>1321</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>1322</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="2" t="s">
         <v>1323</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>1324</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="D4" s="7">
         <v>2024</v>
       </c>
       <c r="F4" s="7" t="s">
+        <v>1325</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>1326</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>1327</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D5" s="7">
         <v>2024</v>
       </c>
       <c r="F5" s="7" t="s">
+        <v>1328</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>1329</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>1330</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>1331</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D6" s="7">
         <v>2024</v>
       </c>
       <c r="F6" s="7" t="s">
+        <v>1331</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>1332</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>1333</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>1334</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="D7" s="7">
         <v>2025</v>
       </c>
       <c r="F7" s="9" t="s">
+        <v>1335</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>1336</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>1337</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>1338</v>
       </c>
     </row>
   </sheetData>
@@ -11988,1231 +11985,1231 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1109</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1110</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>1111</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>1112</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1110</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1113</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>1114</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>1114</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>1115</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>1115</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>1116</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>1116</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>1117</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>1118</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>1118</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>1119</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>1110</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>1111</v>
-      </c>
       <c r="C6" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>1120</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>1110</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>1121</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>1124</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>1118</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>1125</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>1110</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>1111</v>
-      </c>
       <c r="C10" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>1126</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>1110</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>1127</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>1131</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>1132</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>1133</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>1134</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>1135</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>1136</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>1137</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>1138</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>1139</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>1140</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>1141</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>1142</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>1143</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>1144</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>1145</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>1146</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
+        <v>1146</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>1147</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>1148</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>1149</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>1150</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>1151</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>1152</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>1152</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>1153</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>1154</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>1155</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>1131</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>1132</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>1133</v>
-      </c>
       <c r="E22" s="2" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>1135</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>1136</v>
-      </c>
       <c r="E23" s="2" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>1138</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>1139</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>1141</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>1142</v>
-      </c>
       <c r="E25" s="2" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>1144</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>1145</v>
-      </c>
       <c r="E26" s="2" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
+        <v>1146</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>1147</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>1148</v>
-      </c>
       <c r="E27" s="2" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>1150</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>1151</v>
-      </c>
       <c r="E28" s="2" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>1152</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>1153</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>1154</v>
-      </c>
       <c r="E29" s="2" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>1131</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>1132</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>1133</v>
-      </c>
       <c r="E30" s="2" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>1135</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>1136</v>
-      </c>
       <c r="E31" s="2" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>1138</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>1139</v>
-      </c>
       <c r="E32" s="2" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>1141</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>1142</v>
-      </c>
       <c r="E33" s="2" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>1144</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>1145</v>
-      </c>
       <c r="E34" s="2" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>1146</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>1147</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>1148</v>
-      </c>
       <c r="E35" s="2" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>1150</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>1151</v>
-      </c>
       <c r="E36" s="2" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
+        <v>1152</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>1153</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>1132</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>1154</v>
-      </c>
       <c r="E37" s="2" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>1172</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>1173</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>1172</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>1174</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>1175</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>1175</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>1176</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>1177</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>1179</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>1179</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>1180</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
+        <v>1180</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>1180</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>1181</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>1181</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>1182</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
+        <v>1182</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>1182</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>1183</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>1183</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>1184</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>1185</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>1185</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>1186</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>1187</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>1187</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>1188</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>1189</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>1189</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>1190</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>1191</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>1191</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>1192</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>1192</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>1193</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>1193</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>1194</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>1194</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>1195</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>1196</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>1172</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>1173</v>
-      </c>
       <c r="C50" s="2" t="s">
+        <v>1196</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>1197</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>1172</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>1198</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>1172</v>
       </c>
-      <c r="B62" s="2" t="s">
-        <v>1173</v>
-      </c>
       <c r="C62" s="2" t="s">
+        <v>1209</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E62" s="2" t="s">
         <v>1210</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>1172</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>1211</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
     </row>
   </sheetData>
@@ -13233,7 +13230,7 @@
         <v>1106</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
@@ -13244,223 +13241,223 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1224</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>1224</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>1226</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1225</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1227</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>1228</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>1229</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>1230</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>1229</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>1231</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>1232</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>1233</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>1232</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>1234</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>1233</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>1235</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>1236</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>1237</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>1236</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>1238</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>1237</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>1239</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>1240</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>1241</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>1240</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>1242</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>1241</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>1243</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>1244</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>1245</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>1245</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>1246</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>1246</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>1247</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>1247</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>1248</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>1249</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>1248</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>1250</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>1249</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>1251</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>1252</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>1253</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>1252</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>1254</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>1253</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>1255</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>1255</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>1256</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>1257</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>1256</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>1258</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>1257</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>1259</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>1259</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>1260</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>1261</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>1262</v>
-      </c>
       <c r="D11" s="2" t="s">
+        <v>1260</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>1261</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>1262</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>1263</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>1264</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>1265</v>
-      </c>
       <c r="D12" s="2" t="s">
+        <v>1263</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>1264</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>1265</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>1266</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>1267</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>1267</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>1267</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>1268</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>1269</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>1269</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>1269</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>1270</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>1270</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>1270</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>1271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix nexus-e and calliope model labels
</commit_message>
<xml_diff>
--- a/data/dimensions/dimensions.xlsx
+++ b/data/dimensions/dimensions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrianamarcucci/Documents/GitHub/cross/data_model_tmp/data/dimensions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05733BA1-1793-F747-A875-FBDF62103C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B23B1C-339B-B74E-8E20-ED11479578E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41560" yWindow="2020" windowWidth="23500" windowHeight="19000" tabRatio="808" firstSheet="15" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41240" yWindow="2040" windowWidth="23500" windowHeight="19000" tabRatio="808" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="21" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2970" uniqueCount="1650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2970" uniqueCount="1651">
   <si>
     <t>id</t>
   </si>
@@ -5004,6 +5004,9 @@
   </si>
   <si>
     <t>Space heating: Electric heater</t>
+  </si>
+  <si>
+    <t>Calliope</t>
   </si>
 </sst>
 </file>
@@ -5103,7 +5106,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5124,7 +5127,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -15989,7 +15991,7 @@
         <v>1156</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1155</v>
+        <v>1650</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>1157</v>
@@ -16049,7 +16051,7 @@
         <v>1166</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>1167</v>
@@ -16426,7 +16428,7 @@
       <c r="D5" t="s">
         <v>595</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" t="s">
         <v>1625</v>
       </c>
       <c r="F5" t="s">
@@ -17408,7 +17410,7 @@
       <c r="D11" t="s">
         <v>595</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" t="s">
         <v>1625</v>
       </c>
       <c r="F11" t="s">

</xml_diff>

<commit_message>
Fix nexus-e and calliope model labels (#12)
</commit_message>
<xml_diff>
--- a/data/dimensions/dimensions.xlsx
+++ b/data/dimensions/dimensions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrianamarcucci/Documents/GitHub/cross/data_model_tmp/data/dimensions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05733BA1-1793-F747-A875-FBDF62103C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B23B1C-339B-B74E-8E20-ED11479578E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41560" yWindow="2020" windowWidth="23500" windowHeight="19000" tabRatio="808" firstSheet="15" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41240" yWindow="2040" windowWidth="23500" windowHeight="19000" tabRatio="808" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="21" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2970" uniqueCount="1650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2970" uniqueCount="1651">
   <si>
     <t>id</t>
   </si>
@@ -5004,6 +5004,9 @@
   </si>
   <si>
     <t>Space heating: Electric heater</t>
+  </si>
+  <si>
+    <t>Calliope</t>
   </si>
 </sst>
 </file>
@@ -5103,7 +5106,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5124,7 +5127,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -15989,7 +15991,7 @@
         <v>1156</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1155</v>
+        <v>1650</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>1157</v>
@@ -16049,7 +16051,7 @@
         <v>1166</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>1167</v>
@@ -16426,7 +16428,7 @@
       <c r="D5" t="s">
         <v>595</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" t="s">
         <v>1625</v>
       </c>
       <c r="F5" t="s">
@@ -17408,7 +17410,7 @@
       <c r="D11" t="s">
         <v>595</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" t="s">
         <v>1625</v>
       </c>
       <c r="F11" t="s">

</xml_diff>